<commit_message>
Cambio en Proveedores IA
</commit_message>
<xml_diff>
--- a/public/data/Auditoria_Mantenimiento_Generado (28-08).xlsx
+++ b/public/data/Auditoria_Mantenimiento_Generado (28-08).xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8496"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9072"/>
   </bookViews>
   <sheets>
     <sheet name="Auditoría" sheetId="1" r:id="rId1"/>
@@ -921,16 +921,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF00B0F0"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">

</xml_diff>